<commit_message>
E21/E22: cost-per-lead denominators use the MAX(1, …) guard; API test reads the catalog
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wfo8X2RieW62rJiiP3xP73
</commit_message>
<xml_diff>
--- a/samples/fitness-full.xlsx
+++ b/samples/fitness-full.xlsx
@@ -3710,147 +3710,147 @@
         <v>32</v>
       </c>
       <c r="C8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-C35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-C35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>19.2</v>
       </c>
       <c r="D8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-D35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-D35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>19.2</v>
       </c>
       <c r="E8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-E35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-E35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>19.2</v>
       </c>
       <c r="F8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-F35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-F35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>19.2</v>
       </c>
       <c r="G8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-G35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-G35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>19.2</v>
       </c>
       <c r="H8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-H35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-H35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>19.2</v>
       </c>
       <c r="I8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-I35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-I35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>19.2</v>
       </c>
       <c r="J8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-J35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-J35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>19.2</v>
       </c>
       <c r="K8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-K35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-K35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>19.2</v>
       </c>
       <c r="L8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-L35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-L35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>19.2</v>
       </c>
       <c r="M8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-M35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-M35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>19.2</v>
       </c>
       <c r="N8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-N35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-N35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>19.2</v>
       </c>
       <c r="O8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-O35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-O35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>20.16</v>
       </c>
       <c r="P8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-P35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-P35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>20.16</v>
       </c>
       <c r="Q8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-Q35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-Q35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>20.16</v>
       </c>
       <c r="R8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-R35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-R35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>20.16</v>
       </c>
       <c r="S8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-S35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-S35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>20.16</v>
       </c>
       <c r="T8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-T35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-T35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>20.16</v>
       </c>
       <c r="U8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-U35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-U35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>20.16</v>
       </c>
       <c r="V8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-V35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-V35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>20.16</v>
       </c>
       <c r="W8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-W35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-W35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>20.16</v>
       </c>
       <c r="X8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-X35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-X35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>20.16</v>
       </c>
       <c r="Y8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-Y35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-Y35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>20.16</v>
       </c>
       <c r="Z8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-Z35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-Z35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>20.16</v>
       </c>
       <c r="AA8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-AA35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-AA35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>21.168</v>
       </c>
       <c r="AB8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-AB35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-AB35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>21.168</v>
       </c>
       <c r="AC8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-AC35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-AC35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>21.168</v>
       </c>
       <c r="AD8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-AD35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-AD35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>21.168</v>
       </c>
       <c r="AE8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-AE35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-AE35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>21.168</v>
       </c>
       <c r="AF8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-AF35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-AF35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>21.168</v>
       </c>
       <c r="AG8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-AG35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-AG35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>21.168</v>
       </c>
       <c r="AH8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-AH35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-AH35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>21.168</v>
       </c>
       <c r="AI8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-AI35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-AI35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>21.168</v>
       </c>
       <c r="AJ8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-AJ35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-AJ35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>21.168</v>
       </c>
       <c r="AK8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-AK35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-AK35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>21.168</v>
       </c>
       <c r="AL8" s="13" t="n">
-        <f aca="false">IF(Inputs!$E$13=0,0,-AL35/Inputs!$E$13*Inputs!$E$14)</f>
+        <f aca="false">-AL35/MAX(1,Inputs!$E$13)*Inputs!$E$14</f>
         <v>21.168</v>
       </c>
     </row>

</xml_diff>